<commit_message>
screener: relatório de 2026-08-05
</commit_message>
<xml_diff>
--- a/reports/screener_2026-08-05.xlsx
+++ b/reports/screener_2026-08-05.xlsx
@@ -1371,10 +1371,10 @@
         </is>
       </c>
       <c r="AW5" t="n">
-        <v>5.639999866485596</v>
+        <v>5.619999885559082</v>
       </c>
       <c r="AX5" t="n">
-        <v>-14.71631105238386</v>
+        <v>-14.41281066323299</v>
       </c>
       <c r="AY5" t="n">
         <v>-39.50409545018086</v>
@@ -1390,7 +1390,7 @@
       </c>
       <c r="BC5" t="inlineStr">
         <is>
-          <t>sem sinal (-14.7% do topo; Em Baixa)</t>
+          <t>sem sinal (-14.4% do topo; Em Baixa)</t>
         </is>
       </c>
     </row>
@@ -2059,10 +2059,10 @@
         </is>
       </c>
       <c r="AW9" t="n">
-        <v>19.21999931335449</v>
+        <v>18.85000038146973</v>
       </c>
       <c r="AX9" t="n">
-        <v>-16.54525760371704</v>
+        <v>-14.90715866883865</v>
       </c>
       <c r="AY9" t="n">
         <v>-54.13720844041888</v>
@@ -2078,7 +2078,7 @@
       </c>
       <c r="BC9" t="inlineStr">
         <is>
-          <t>sem sinal (-16.5% do topo; Em Baixa)</t>
+          <t>sem sinal (-14.9% do topo; Em Baixa)</t>
         </is>
       </c>
     </row>
@@ -2409,7 +2409,7 @@
       </c>
       <c r="AV11" t="inlineStr">
         <is>
-          <t>Em Alta</t>
+          <t>Lateral</t>
         </is>
       </c>
       <c r="AW11" t="n">
@@ -2763,7 +2763,7 @@
       <c r="AU13" t="inlineStr"/>
       <c r="AV13" t="inlineStr">
         <is>
-          <t>Em Baixa</t>
+          <t>Lateral</t>
         </is>
       </c>
       <c r="AW13" t="n">
@@ -2786,7 +2786,7 @@
       </c>
       <c r="BC13" t="inlineStr">
         <is>
-          <t>sem sinal (-3.6% do topo; Em Baixa)</t>
+          <t>sem sinal (-3.6% do topo; Lateral)</t>
         </is>
       </c>
     </row>
@@ -2944,10 +2944,10 @@
         </is>
       </c>
       <c r="AW14" t="n">
-        <v>13</v>
+        <v>12.72999954223633</v>
       </c>
       <c r="AX14" t="n">
-        <v>-14.30768966674805</v>
+        <v>-12.4901748318072</v>
       </c>
       <c r="AY14" t="n">
         <v>-32.85678377733036</v>
@@ -2963,7 +2963,7 @@
       </c>
       <c r="BC14" t="inlineStr">
         <is>
-          <t>sem sinal (-14.3% do topo; Em Baixa)</t>
+          <t>sem sinal (-12.5% do topo; Em Baixa)</t>
         </is>
       </c>
     </row>
@@ -3117,10 +3117,10 @@
         </is>
       </c>
       <c r="AW15" t="n">
-        <v>43.04999923706055</v>
+        <v>43.41999816894531</v>
       </c>
       <c r="AX15" t="n">
-        <v>-1.277582454837922</v>
+        <v>-2.118835116863982</v>
       </c>
       <c r="AY15" t="n">
         <v>-13.54395936495905</v>
@@ -3136,7 +3136,7 @@
       </c>
       <c r="BC15" t="inlineStr">
         <is>
-          <t>sem sinal (-1.3% do topo; Em Alta)</t>
+          <t>sem sinal (-2.1% do topo; Em Alta)</t>
         </is>
       </c>
     </row>
@@ -4336,10 +4336,10 @@
         </is>
       </c>
       <c r="AW22" t="n">
-        <v>48.70000076293945</v>
+        <v>49.04000091552734</v>
       </c>
       <c r="AX22" t="n">
-        <v>-1.129361865388501</v>
+        <v>-1.814843745989081</v>
       </c>
       <c r="AY22" t="n">
         <v>-11.83384458058885</v>
@@ -4355,7 +4355,7 @@
       </c>
       <c r="BC22" t="inlineStr">
         <is>
-          <t>sem sinal (-1.1% do topo; Em Alta)</t>
+          <t>sem sinal (-1.8% do topo; Em Alta)</t>
         </is>
       </c>
     </row>
@@ -5036,10 +5036,10 @@
         </is>
       </c>
       <c r="AW26" t="n">
-        <v>6.579999923706055</v>
+        <v>6.550000190734863</v>
       </c>
       <c r="AX26" t="n">
-        <v>-3.49544105988292</v>
+        <v>-3.053439393562163</v>
       </c>
       <c r="AY26" t="n">
         <v>-39.52381043207078</v>
@@ -5055,7 +5055,7 @@
       </c>
       <c r="BC26" t="inlineStr">
         <is>
-          <t>sem sinal (-3.5% do topo; Em Baixa)</t>
+          <t>sem sinal (-3.1% do topo; Em Baixa)</t>
         </is>
       </c>
     </row>
@@ -5521,7 +5521,7 @@
         <v>-2.713682693188602</v>
       </c>
       <c r="AY29" t="n">
-        <v>-39.51925229062647</v>
+        <v>-39.5192605242667</v>
       </c>
       <c r="AZ29" t="b">
         <v>1</v>
@@ -6217,7 +6217,7 @@
         <v>-3.517688651440576</v>
       </c>
       <c r="AY33" t="n">
-        <v>-12.46353572253916</v>
+        <v>-12.46351675410393</v>
       </c>
       <c r="AZ33" t="b">
         <v>1</v>
@@ -6376,7 +6376,7 @@
       <c r="AU34" t="inlineStr"/>
       <c r="AV34" t="inlineStr">
         <is>
-          <t>Em Alta</t>
+          <t>Lateral</t>
         </is>
       </c>
       <c r="AW34" t="n">
@@ -6399,7 +6399,7 @@
       </c>
       <c r="BC34" t="inlineStr">
         <is>
-          <t>sem sinal (-2.2% do topo; Em Alta)</t>
+          <t>sem sinal (-2.2% do topo; Lateral)</t>
         </is>
       </c>
     </row>
@@ -6726,10 +6726,10 @@
         </is>
       </c>
       <c r="AW36" t="n">
-        <v>29.75</v>
+        <v>29.73999977111816</v>
       </c>
       <c r="AX36" t="n">
-        <v>-2.285715311515235</v>
+        <v>-2.252858377438904</v>
       </c>
       <c r="AY36" t="n">
         <v>-17.59775069846685</v>
@@ -6903,10 +6903,10 @@
         </is>
       </c>
       <c r="AW37" t="n">
-        <v>2.339999914169312</v>
+        <v>2.329999923706055</v>
       </c>
       <c r="AX37" t="n">
-        <v>-3.418800283779255</v>
+        <v>-3.004289078750577</v>
       </c>
       <c r="AY37" t="n">
         <v>-52.18694930098489</v>
@@ -6922,7 +6922,7 @@
       </c>
       <c r="BC37" t="inlineStr">
         <is>
-          <t>sem sinal (-3.4% do topo; Em Baixa)</t>
+          <t>sem sinal (-3.0% do topo; Em Baixa)</t>
         </is>
       </c>
     </row>
@@ -7076,10 +7076,10 @@
         </is>
       </c>
       <c r="AW38" t="n">
-        <v>3.980000019073486</v>
+        <v>4.03000020980835</v>
       </c>
       <c r="AX38" t="n">
-        <v>-0.7537681217588132</v>
+        <v>-1.98511558212644</v>
       </c>
       <c r="AY38" t="n">
         <v>-47.92224740248528</v>
@@ -7095,7 +7095,7 @@
       </c>
       <c r="BC38" t="inlineStr">
         <is>
-          <t>sem sinal (-0.8% do topo; Lateral)</t>
+          <t>sem sinal (-2.0% do topo; Lateral)</t>
         </is>
       </c>
     </row>
@@ -7955,7 +7955,7 @@
         <v>-0.5080771590812438</v>
       </c>
       <c r="AY43" t="n">
-        <v>-19.64053433208342</v>
+        <v>-19.64052806350488</v>
       </c>
       <c r="AZ43" t="b">
         <v>1</v>
@@ -8466,7 +8466,7 @@
         <v>-4.020742883737105</v>
       </c>
       <c r="AY46" t="n">
-        <v>-14.35606196730216</v>
+        <v>-14.3560541194689</v>
       </c>
       <c r="AZ46" t="b">
         <v>1</v>
@@ -8979,10 +8979,10 @@
         </is>
       </c>
       <c r="AW49" t="n">
-        <v>11.27999973297119</v>
+        <v>11.34000015258789</v>
       </c>
       <c r="AX49" t="n">
-        <v>0</v>
+        <v>-0.5291042223046771</v>
       </c>
       <c r="AY49" t="n">
         <v>-15.4147281673955</v>
@@ -8998,7 +8998,7 @@
       </c>
       <c r="BC49" t="inlineStr">
         <is>
-          <t>sem sinal (+0.0% do topo; Em Alta)</t>
+          <t>sem sinal (-0.5% do topo; Em Alta)</t>
         </is>
       </c>
     </row>
@@ -9156,10 +9156,10 @@
         </is>
       </c>
       <c r="AW50" t="n">
-        <v>16.3700008392334</v>
+        <v>16.1200008392334</v>
       </c>
       <c r="AX50" t="n">
-        <v>-14.84423417392992</v>
+        <v>-13.52358030617676</v>
       </c>
       <c r="AY50" t="n">
         <v>-34.85117715011583</v>
@@ -9175,7 +9175,7 @@
       </c>
       <c r="BC50" t="inlineStr">
         <is>
-          <t>sem sinal (-14.8% do topo; Em Baixa)</t>
+          <t>sem sinal (-13.5% do topo; Em Baixa)</t>
         </is>
       </c>
     </row>
@@ -9506,14 +9506,14 @@
       <c r="AU52" t="inlineStr"/>
       <c r="AV52" t="inlineStr">
         <is>
-          <t>Lateral</t>
+          <t>Em Alta</t>
         </is>
       </c>
       <c r="AW52" t="n">
-        <v>43.09999847412109</v>
+        <v>43.31999969482422</v>
       </c>
       <c r="AX52" t="n">
-        <v>-0.1856102533401627</v>
+        <v>-0.6925190193304398</v>
       </c>
       <c r="AY52" t="n">
         <v>-27.87197279000151</v>
@@ -9529,7 +9529,7 @@
       </c>
       <c r="BC52" t="inlineStr">
         <is>
-          <t>sem sinal (-0.2% do topo; Lateral)</t>
+          <t>sem sinal (-0.7% do topo; Em Alta)</t>
         </is>
       </c>
     </row>
@@ -10500,13 +10500,13 @@
         </is>
       </c>
       <c r="AW58" t="n">
-        <v>43.63000106811523</v>
+        <v>43.61150741577148</v>
       </c>
       <c r="AX58" t="n">
-        <v>-3.506767262291599</v>
+        <v>-3.465848880756128</v>
       </c>
       <c r="AY58" t="n">
-        <v>-13.58724744836764</v>
+        <v>-13.55060950604702</v>
       </c>
       <c r="AZ58" t="b">
         <v>1</v>
@@ -10669,7 +10669,7 @@
       <c r="AU59" t="inlineStr"/>
       <c r="AV59" t="inlineStr">
         <is>
-          <t>Em Baixa</t>
+          <t>Lateral</t>
         </is>
       </c>
       <c r="AW59" t="n">
@@ -10692,7 +10692,7 @@
       </c>
       <c r="BC59" t="inlineStr">
         <is>
-          <t>sem sinal (-2.7% do topo; Em Baixa)</t>
+          <t>sem sinal (-2.7% do topo; Lateral)</t>
         </is>
       </c>
     </row>
@@ -10852,7 +10852,7 @@
         <v>-0.9501178501326923</v>
       </c>
       <c r="AY60" t="n">
-        <v>-14.40870028403989</v>
+        <v>-14.40870883002358</v>
       </c>
       <c r="AZ60" t="b">
         <v>1</v>
@@ -13006,10 +13006,10 @@
         </is>
       </c>
       <c r="AW5" t="n">
-        <v>5.639999866485596</v>
+        <v>5.619999885559082</v>
       </c>
       <c r="AX5" t="n">
-        <v>-14.71631105238386</v>
+        <v>-14.41281066323299</v>
       </c>
       <c r="AY5" t="n">
         <v>-39.50409545018086</v>
@@ -13025,7 +13025,7 @@
       </c>
       <c r="BC5" t="inlineStr">
         <is>
-          <t>sem sinal (-14.7% do topo; Em Baixa)</t>
+          <t>sem sinal (-14.4% do topo; Em Baixa)</t>
         </is>
       </c>
     </row>
@@ -13694,10 +13694,10 @@
         </is>
       </c>
       <c r="AW9" t="n">
-        <v>19.21999931335449</v>
+        <v>18.85000038146973</v>
       </c>
       <c r="AX9" t="n">
-        <v>-16.54525760371704</v>
+        <v>-14.90715866883865</v>
       </c>
       <c r="AY9" t="n">
         <v>-54.13720844041888</v>
@@ -13713,7 +13713,7 @@
       </c>
       <c r="BC9" t="inlineStr">
         <is>
-          <t>sem sinal (-16.5% do topo; Em Baixa)</t>
+          <t>sem sinal (-14.9% do topo; Em Baixa)</t>
         </is>
       </c>
     </row>
@@ -14044,7 +14044,7 @@
       </c>
       <c r="AV11" t="inlineStr">
         <is>
-          <t>Em Alta</t>
+          <t>Lateral</t>
         </is>
       </c>
       <c r="AW11" t="n">
@@ -14398,7 +14398,7 @@
       <c r="AU13" t="inlineStr"/>
       <c r="AV13" t="inlineStr">
         <is>
-          <t>Em Baixa</t>
+          <t>Lateral</t>
         </is>
       </c>
       <c r="AW13" t="n">
@@ -14421,7 +14421,7 @@
       </c>
       <c r="BC13" t="inlineStr">
         <is>
-          <t>sem sinal (-3.6% do topo; Em Baixa)</t>
+          <t>sem sinal (-3.6% do topo; Lateral)</t>
         </is>
       </c>
     </row>
@@ -14579,10 +14579,10 @@
         </is>
       </c>
       <c r="AW14" t="n">
-        <v>13</v>
+        <v>12.72999954223633</v>
       </c>
       <c r="AX14" t="n">
-        <v>-14.30768966674805</v>
+        <v>-12.4901748318072</v>
       </c>
       <c r="AY14" t="n">
         <v>-32.85678377733036</v>
@@ -14598,7 +14598,7 @@
       </c>
       <c r="BC14" t="inlineStr">
         <is>
-          <t>sem sinal (-14.3% do topo; Em Baixa)</t>
+          <t>sem sinal (-12.5% do topo; Em Baixa)</t>
         </is>
       </c>
     </row>
@@ -14752,10 +14752,10 @@
         </is>
       </c>
       <c r="AW15" t="n">
-        <v>43.04999923706055</v>
+        <v>43.41999816894531</v>
       </c>
       <c r="AX15" t="n">
-        <v>-1.277582454837922</v>
+        <v>-2.118835116863982</v>
       </c>
       <c r="AY15" t="n">
         <v>-13.54395936495905</v>
@@ -14771,7 +14771,7 @@
       </c>
       <c r="BC15" t="inlineStr">
         <is>
-          <t>sem sinal (-1.3% do topo; Em Alta)</t>
+          <t>sem sinal (-2.1% do topo; Em Alta)</t>
         </is>
       </c>
     </row>
@@ -15971,10 +15971,10 @@
         </is>
       </c>
       <c r="AW22" t="n">
-        <v>48.70000076293945</v>
+        <v>49.04000091552734</v>
       </c>
       <c r="AX22" t="n">
-        <v>-1.129361865388501</v>
+        <v>-1.814843745989081</v>
       </c>
       <c r="AY22" t="n">
         <v>-11.83384458058885</v>
@@ -15990,7 +15990,7 @@
       </c>
       <c r="BC22" t="inlineStr">
         <is>
-          <t>sem sinal (-1.1% do topo; Em Alta)</t>
+          <t>sem sinal (-1.8% do topo; Em Alta)</t>
         </is>
       </c>
     </row>
@@ -16838,10 +16838,10 @@
         </is>
       </c>
       <c r="AW27" t="n">
-        <v>6.579999923706055</v>
+        <v>6.550000190734863</v>
       </c>
       <c r="AX27" t="n">
-        <v>-3.49544105988292</v>
+        <v>-3.053439393562163</v>
       </c>
       <c r="AY27" t="n">
         <v>-39.52381043207078</v>
@@ -16857,7 +16857,7 @@
       </c>
       <c r="BC27" t="inlineStr">
         <is>
-          <t>sem sinal (-3.5% do topo; Em Baixa)</t>
+          <t>sem sinal (-3.1% do topo; Em Baixa)</t>
         </is>
       </c>
     </row>
@@ -17323,7 +17323,7 @@
         <v>-2.713682693188602</v>
       </c>
       <c r="AY30" t="n">
-        <v>-39.51925229062647</v>
+        <v>-39.5192605242667</v>
       </c>
       <c r="AZ30" t="b">
         <v>1</v>
@@ -18019,7 +18019,7 @@
         <v>-3.517688651440576</v>
       </c>
       <c r="AY34" t="n">
-        <v>-12.46353572253916</v>
+        <v>-12.46351675410393</v>
       </c>
       <c r="AZ34" t="b">
         <v>1</v>
@@ -18178,7 +18178,7 @@
       <c r="AU35" t="inlineStr"/>
       <c r="AV35" t="inlineStr">
         <is>
-          <t>Em Alta</t>
+          <t>Lateral</t>
         </is>
       </c>
       <c r="AW35" t="n">
@@ -18201,7 +18201,7 @@
       </c>
       <c r="BC35" t="inlineStr">
         <is>
-          <t>sem sinal (-2.2% do topo; Em Alta)</t>
+          <t>sem sinal (-2.2% do topo; Lateral)</t>
         </is>
       </c>
     </row>
@@ -18528,10 +18528,10 @@
         </is>
       </c>
       <c r="AW37" t="n">
-        <v>29.75</v>
+        <v>29.73999977111816</v>
       </c>
       <c r="AX37" t="n">
-        <v>-2.285715311515235</v>
+        <v>-2.252858377438904</v>
       </c>
       <c r="AY37" t="n">
         <v>-17.59775069846685</v>
@@ -18705,10 +18705,10 @@
         </is>
       </c>
       <c r="AW38" t="n">
-        <v>2.339999914169312</v>
+        <v>2.329999923706055</v>
       </c>
       <c r="AX38" t="n">
-        <v>-3.418800283779255</v>
+        <v>-3.004289078750577</v>
       </c>
       <c r="AY38" t="n">
         <v>-52.18694930098489</v>
@@ -18724,7 +18724,7 @@
       </c>
       <c r="BC38" t="inlineStr">
         <is>
-          <t>sem sinal (-3.4% do topo; Em Baixa)</t>
+          <t>sem sinal (-3.0% do topo; Em Baixa)</t>
         </is>
       </c>
     </row>
@@ -18878,10 +18878,10 @@
         </is>
       </c>
       <c r="AW39" t="n">
-        <v>3.980000019073486</v>
+        <v>4.03000020980835</v>
       </c>
       <c r="AX39" t="n">
-        <v>-0.7537681217588132</v>
+        <v>-1.98511558212644</v>
       </c>
       <c r="AY39" t="n">
         <v>-47.92224740248528</v>
@@ -18897,7 +18897,7 @@
       </c>
       <c r="BC39" t="inlineStr">
         <is>
-          <t>sem sinal (-0.8% do topo; Lateral)</t>
+          <t>sem sinal (-2.0% do topo; Lateral)</t>
         </is>
       </c>
     </row>
@@ -19757,7 +19757,7 @@
         <v>-0.5080771590812438</v>
       </c>
       <c r="AY44" t="n">
-        <v>-19.64053433208342</v>
+        <v>-19.64052806350488</v>
       </c>
       <c r="AZ44" t="b">
         <v>1</v>
@@ -20268,7 +20268,7 @@
         <v>-4.020742883737105</v>
       </c>
       <c r="AY47" t="n">
-        <v>-14.35606196730216</v>
+        <v>-14.3560541194689</v>
       </c>
       <c r="AZ47" t="b">
         <v>1</v>
@@ -20781,10 +20781,10 @@
         </is>
       </c>
       <c r="AW50" t="n">
-        <v>11.27999973297119</v>
+        <v>11.34000015258789</v>
       </c>
       <c r="AX50" t="n">
-        <v>0</v>
+        <v>-0.5291042223046771</v>
       </c>
       <c r="AY50" t="n">
         <v>-15.4147281673955</v>
@@ -20800,7 +20800,7 @@
       </c>
       <c r="BC50" t="inlineStr">
         <is>
-          <t>sem sinal (+0.0% do topo; Em Alta)</t>
+          <t>sem sinal (-0.5% do topo; Em Alta)</t>
         </is>
       </c>
     </row>
@@ -20958,10 +20958,10 @@
         </is>
       </c>
       <c r="AW51" t="n">
-        <v>16.3700008392334</v>
+        <v>16.1200008392334</v>
       </c>
       <c r="AX51" t="n">
-        <v>-14.84423417392992</v>
+        <v>-13.52358030617676</v>
       </c>
       <c r="AY51" t="n">
         <v>-34.85117715011583</v>
@@ -20977,7 +20977,7 @@
       </c>
       <c r="BC51" t="inlineStr">
         <is>
-          <t>sem sinal (-14.8% do topo; Em Baixa)</t>
+          <t>sem sinal (-13.5% do topo; Em Baixa)</t>
         </is>
       </c>
     </row>
@@ -21308,14 +21308,14 @@
       <c r="AU53" t="inlineStr"/>
       <c r="AV53" t="inlineStr">
         <is>
-          <t>Lateral</t>
+          <t>Em Alta</t>
         </is>
       </c>
       <c r="AW53" t="n">
-        <v>43.09999847412109</v>
+        <v>43.31999969482422</v>
       </c>
       <c r="AX53" t="n">
-        <v>-0.1856102533401627</v>
+        <v>-0.6925190193304398</v>
       </c>
       <c r="AY53" t="n">
         <v>-27.87197279000151</v>
@@ -21331,7 +21331,7 @@
       </c>
       <c r="BC53" t="inlineStr">
         <is>
-          <t>sem sinal (-0.2% do topo; Lateral)</t>
+          <t>sem sinal (-0.7% do topo; Em Alta)</t>
         </is>
       </c>
     </row>
@@ -22302,13 +22302,13 @@
         </is>
       </c>
       <c r="AW59" t="n">
-        <v>43.63000106811523</v>
+        <v>43.61150741577148</v>
       </c>
       <c r="AX59" t="n">
-        <v>-3.506767262291599</v>
+        <v>-3.465848880756128</v>
       </c>
       <c r="AY59" t="n">
-        <v>-13.58724744836764</v>
+        <v>-13.55060950604702</v>
       </c>
       <c r="AZ59" t="b">
         <v>1</v>
@@ -22471,7 +22471,7 @@
       <c r="AU60" t="inlineStr"/>
       <c r="AV60" t="inlineStr">
         <is>
-          <t>Em Baixa</t>
+          <t>Lateral</t>
         </is>
       </c>
       <c r="AW60" t="n">
@@ -22494,7 +22494,7 @@
       </c>
       <c r="BC60" t="inlineStr">
         <is>
-          <t>sem sinal (-2.7% do topo; Em Baixa)</t>
+          <t>sem sinal (-2.7% do topo; Lateral)</t>
         </is>
       </c>
     </row>
@@ -22654,7 +22654,7 @@
         <v>-0.9501178501326923</v>
       </c>
       <c r="AY61" t="n">
-        <v>-14.40870028403989</v>
+        <v>-14.40870883002358</v>
       </c>
       <c r="AZ61" t="b">
         <v>1</v>
@@ -23996,7 +23996,7 @@
         <v>-1.302573977731003</v>
       </c>
       <c r="AY69" t="n">
-        <v>-15.92981174353384</v>
+        <v>-15.92983151621281</v>
       </c>
       <c r="AZ69" t="b">
         <v>0</v>
@@ -24163,10 +24163,10 @@
         </is>
       </c>
       <c r="AW70" t="n">
-        <v>76.08999633789062</v>
+        <v>76.27999877929688</v>
       </c>
       <c r="AX70" t="n">
-        <v>0.2891329100952689</v>
+        <v>0.03932718901014098</v>
       </c>
       <c r="AY70" t="n">
         <v>-16.71033041805866</v>
@@ -24336,10 +24336,10 @@
         </is>
       </c>
       <c r="AW71" t="n">
-        <v>30.3700008392334</v>
+        <v>30.34000015258789</v>
       </c>
       <c r="AX71" t="n">
-        <v>-7.770828268476048</v>
+        <v>-7.679630560276429</v>
       </c>
       <c r="AY71" t="n">
         <v>-20.69199954808616</v>
@@ -24355,7 +24355,7 @@
       </c>
       <c r="BC71" t="inlineStr">
         <is>
-          <t>sem sinal (-7.8% do topo; Em Baixa)</t>
+          <t>sem sinal (-7.7% do topo; Em Baixa)</t>
         </is>
       </c>
     </row>
@@ -24497,10 +24497,10 @@
         </is>
       </c>
       <c r="AW72" t="n">
-        <v>21.27000045776367</v>
+        <v>21.35000038146973</v>
       </c>
       <c r="AX72" t="n">
-        <v>-1.316411286410224</v>
+        <v>-1.686185498450943</v>
       </c>
       <c r="AY72" t="n">
         <v>-23.79046311986899</v>
@@ -24516,7 +24516,7 @@
       </c>
       <c r="BC72" t="inlineStr">
         <is>
-          <t>sem sinal (-1.3% do topo; Em Alta)</t>
+          <t>sem sinal (-1.7% do topo; Em Alta)</t>
         </is>
       </c>
     </row>
@@ -24664,10 +24664,10 @@
         </is>
       </c>
       <c r="AW73" t="n">
-        <v>4.070000171661377</v>
+        <v>3.990000009536743</v>
       </c>
       <c r="AX73" t="n">
-        <v>-4.422605876297203</v>
+        <v>-2.506263268008835</v>
       </c>
       <c r="AY73" t="n">
         <v>-19.0219927402037</v>
@@ -24683,7 +24683,7 @@
       </c>
       <c r="BC73" t="inlineStr">
         <is>
-          <t>sem sinal (-4.4% do topo; Em Baixa)</t>
+          <t>sem sinal (-2.5% do topo; Em Baixa)</t>
         </is>
       </c>
     </row>
@@ -24817,7 +24817,7 @@
       <c r="AU74" t="inlineStr"/>
       <c r="AV74" t="inlineStr">
         <is>
-          <t>Em Baixa</t>
+          <t>Lateral</t>
         </is>
       </c>
       <c r="AW74" t="n">
@@ -24840,7 +24840,7 @@
       </c>
       <c r="BC74" t="inlineStr">
         <is>
-          <t>sem sinal (-5.3% do topo; Em Baixa)</t>
+          <t>sem sinal (-5.3% do topo; Lateral)</t>
         </is>
       </c>
     </row>
@@ -25332,7 +25332,7 @@
       <c r="AU77" t="inlineStr"/>
       <c r="AV77" t="inlineStr">
         <is>
-          <t>Lateral</t>
+          <t>Em Baixa</t>
         </is>
       </c>
       <c r="AW77" t="n">
@@ -25355,7 +25355,7 @@
       </c>
       <c r="BC77" t="inlineStr">
         <is>
-          <t>sem sinal (-10.4% do topo; Lateral)</t>
+          <t>sem sinal (-10.4% do topo; Em Baixa)</t>
         </is>
       </c>
     </row>
@@ -26087,7 +26087,7 @@
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>Rompimento</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="K82" t="n">
@@ -26194,21 +26194,17 @@
       </c>
       <c r="AS82" t="inlineStr"/>
       <c r="AT82" t="inlineStr"/>
-      <c r="AU82" t="inlineStr">
-        <is>
-          <t>Rompimento</t>
-        </is>
-      </c>
+      <c r="AU82" t="inlineStr"/>
       <c r="AV82" t="inlineStr">
         <is>
           <t>Em Alta</t>
         </is>
       </c>
       <c r="AW82" t="n">
-        <v>3.519999980926514</v>
+        <v>3.559999942779541</v>
       </c>
       <c r="AX82" t="n">
-        <v>0.2840906397000742</v>
+        <v>-0.8426958391001382</v>
       </c>
       <c r="AY82" t="n">
         <v>-43.96825611876666</v>
@@ -26217,14 +26213,14 @@
         <v>0</v>
       </c>
       <c r="BA82" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BB82" t="b">
         <v>0</v>
       </c>
       <c r="BC82" t="inlineStr">
         <is>
-          <t>Rompimento</t>
+          <t>sem sinal (-0.8% do topo; Em Alta)</t>
         </is>
       </c>
     </row>
@@ -26262,7 +26258,7 @@
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>Rompimento</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="K83" t="n">
@@ -26363,21 +26359,17 @@
       </c>
       <c r="AS83" t="inlineStr"/>
       <c r="AT83" t="inlineStr"/>
-      <c r="AU83" t="inlineStr">
-        <is>
-          <t>Rompimento</t>
-        </is>
-      </c>
+      <c r="AU83" t="inlineStr"/>
       <c r="AV83" t="inlineStr">
         <is>
           <t>Em Baixa</t>
         </is>
       </c>
       <c r="AW83" t="n">
-        <v>21.85000038146973</v>
+        <v>22</v>
       </c>
       <c r="AX83" t="n">
-        <v>0.09153527420819874</v>
+        <v>-0.5909052762118283</v>
       </c>
       <c r="AY83" t="n">
         <v>-14.67030216407054</v>
@@ -26386,14 +26378,14 @@
         <v>0</v>
       </c>
       <c r="BA83" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BB83" t="b">
         <v>0</v>
       </c>
       <c r="BC83" t="inlineStr">
         <is>
-          <t>Rompimento</t>
+          <t>sem sinal (-0.6% do topo; Em Baixa)</t>
         </is>
       </c>
     </row>
@@ -26543,10 +26535,10 @@
         </is>
       </c>
       <c r="AW84" t="n">
-        <v>60.54000091552734</v>
+        <v>60.84999847412109</v>
       </c>
       <c r="AX84" t="n">
-        <v>-3.452263166470892</v>
+        <v>-3.944121234780862</v>
       </c>
       <c r="AY84" t="n">
         <v>-19.90956690277227</v>
@@ -26562,7 +26554,7 @@
       </c>
       <c r="BC84" t="inlineStr">
         <is>
-          <t>sem sinal (-3.5% do topo; Em Alta)</t>
+          <t>sem sinal (-3.9% do topo; Em Alta)</t>
         </is>
       </c>
     </row>
@@ -26863,10 +26855,10 @@
         </is>
       </c>
       <c r="AW86" t="n">
-        <v>0.1599999964237213</v>
+        <v>0.1700000017881393</v>
       </c>
       <c r="AX86" t="n">
-        <v>0</v>
+        <v>-5.882356034843117</v>
       </c>
       <c r="AY86" t="n">
         <v>-99.17440658744904</v>
@@ -26882,7 +26874,7 @@
       </c>
       <c r="BC86" t="inlineStr">
         <is>
-          <t>sem sinal (+0.0% do topo; Em Baixa)</t>
+          <t>sem sinal (-5.9% do topo; Em Baixa)</t>
         </is>
       </c>
     </row>
@@ -27867,10 +27859,10 @@
         </is>
       </c>
       <c r="AW92" t="n">
-        <v>66.26999664306641</v>
+        <v>66.09999847412109</v>
       </c>
       <c r="AX92" t="n">
-        <v>-3.561184420100938</v>
+        <v>-3.313159874831761</v>
       </c>
       <c r="AY92" t="n">
         <v>-5.76526078591314</v>
@@ -27886,7 +27878,7 @@
       </c>
       <c r="BC92" t="inlineStr">
         <is>
-          <t>sem sinal (-3.6% do topo; Em Alta)</t>
+          <t>sem sinal (-3.3% do topo; Em Alta)</t>
         </is>
       </c>
     </row>
@@ -28553,10 +28545,10 @@
         </is>
       </c>
       <c r="AW96" t="n">
-        <v>21.07999992370605</v>
+        <v>21.17000007629395</v>
       </c>
       <c r="AX96" t="n">
-        <v>-3.889941640379546</v>
+        <v>-4.298534927409481</v>
       </c>
       <c r="AY96" t="n">
         <v>-19.35852192104358</v>
@@ -28572,7 +28564,7 @@
       </c>
       <c r="BC96" t="inlineStr">
         <is>
-          <t>sem sinal (-3.9% do topo; Lateral)</t>
+          <t>sem sinal (-4.3% do topo; Lateral)</t>
         </is>
       </c>
     </row>
@@ -29207,10 +29199,10 @@
         </is>
       </c>
       <c r="AW100" t="n">
-        <v>8.710000038146973</v>
+        <v>8.659999847412109</v>
       </c>
       <c r="AX100" t="n">
-        <v>-0.5740550001823053</v>
+        <v>0</v>
       </c>
       <c r="AY100" t="n">
         <v>-18.43808159694287</v>
@@ -29226,7 +29218,7 @@
       </c>
       <c r="BC100" t="inlineStr">
         <is>
-          <t>sem sinal (-0.6% do topo; Em Baixa)</t>
+          <t>sem sinal (+0.0% do topo; Em Baixa)</t>
         </is>
       </c>
     </row>
@@ -29549,10 +29541,10 @@
         </is>
       </c>
       <c r="AW102" t="n">
-        <v>32.43999862670898</v>
+        <v>32.27000045776367</v>
       </c>
       <c r="AX102" t="n">
-        <v>-7.12083712617817</v>
+        <v>-6.631550252991147</v>
       </c>
       <c r="AY102" t="n">
         <v>-22.38033148894612</v>
@@ -29568,7 +29560,7 @@
       </c>
       <c r="BC102" t="inlineStr">
         <is>
-          <t>sem sinal (-7.1% do topo; Em Baixa)</t>
+          <t>sem sinal (-6.6% do topo; Em Baixa)</t>
         </is>
       </c>
     </row>
@@ -32111,10 +32103,10 @@
         </is>
       </c>
       <c r="AW118" t="n">
-        <v>6.940000057220459</v>
+        <v>6.829999923706055</v>
       </c>
       <c r="AX118" t="n">
-        <v>-15.99423810320502</v>
+        <v>-14.64128859693144</v>
       </c>
       <c r="AY118" t="n">
         <v>-57.6923074261264</v>
@@ -32130,7 +32122,7 @@
       </c>
       <c r="BC118" t="inlineStr">
         <is>
-          <t>sem sinal (-16.0% do topo; Em Baixa)</t>
+          <t>sem sinal (-14.6% do topo; Em Baixa)</t>
         </is>
       </c>
     </row>
@@ -32170,7 +32162,7 @@
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>Rompimento</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="K119" t="n">
@@ -32277,21 +32269,17 @@
       </c>
       <c r="AS119" t="inlineStr"/>
       <c r="AT119" t="inlineStr"/>
-      <c r="AU119" t="inlineStr">
-        <is>
-          <t>Rompimento</t>
-        </is>
-      </c>
+      <c r="AU119" t="inlineStr"/>
       <c r="AV119" t="inlineStr">
         <is>
           <t>Em Alta</t>
         </is>
       </c>
       <c r="AW119" t="n">
-        <v>18.23999977111816</v>
+        <v>18.25</v>
       </c>
       <c r="AX119" t="n">
-        <v>0.05482581692610733</v>
+        <v>0</v>
       </c>
       <c r="AY119" t="n">
         <v>-14.11764705882353</v>
@@ -32300,14 +32288,14 @@
         <v>0</v>
       </c>
       <c r="BA119" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BB119" t="b">
         <v>0</v>
       </c>
       <c r="BC119" t="inlineStr">
         <is>
-          <t>Rompimento</t>
+          <t>sem sinal (+0.0% do topo; Em Alta)</t>
         </is>
       </c>
     </row>
@@ -32789,10 +32777,10 @@
         </is>
       </c>
       <c r="AW122" t="n">
-        <v>14.27999973297119</v>
+        <v>14.4399995803833</v>
       </c>
       <c r="AX122" t="n">
-        <v>-1.120447131680857</v>
+        <v>-2.21606443298612</v>
       </c>
       <c r="AY122" t="n">
         <v>-18.51651739090506</v>
@@ -32808,7 +32796,7 @@
       </c>
       <c r="BC122" t="inlineStr">
         <is>
-          <t>sem sinal (-1.1% do topo; Em Alta)</t>
+          <t>sem sinal (-2.2% do topo; Em Alta)</t>
         </is>
       </c>
     </row>
@@ -33709,10 +33697,10 @@
         </is>
       </c>
       <c r="AW128" t="n">
-        <v>0.3300000131130219</v>
+        <v>0.3100000023841858</v>
       </c>
       <c r="AX128" t="n">
-        <v>-15.15151816185063</v>
+        <v>-9.677419664956521</v>
       </c>
       <c r="AY128" t="n">
         <v>-80.5555562454241</v>
@@ -33728,7 +33716,7 @@
       </c>
       <c r="BC128" t="inlineStr">
         <is>
-          <t>sem sinal (-15.2% do topo; Em Baixa)</t>
+          <t>sem sinal (-9.7% do topo; Em Baixa)</t>
         </is>
       </c>
     </row>
@@ -33874,7 +33862,7 @@
       <c r="AU129" t="inlineStr"/>
       <c r="AV129" t="inlineStr">
         <is>
-          <t>Lateral</t>
+          <t>Em Alta</t>
         </is>
       </c>
       <c r="AW129" t="n">
@@ -33897,7 +33885,7 @@
       </c>
       <c r="BC129" t="inlineStr">
         <is>
-          <t>sem sinal (-1.9% do topo; Lateral)</t>
+          <t>sem sinal (-1.9% do topo; Em Alta)</t>
         </is>
       </c>
     </row>
@@ -34202,10 +34190,10 @@
         </is>
       </c>
       <c r="AW131" t="n">
-        <v>12.31999969482422</v>
+        <v>12.3100004196167</v>
       </c>
       <c r="AX131" t="n">
-        <v>-8.441558341027754</v>
+        <v>-8.367186446266416</v>
       </c>
       <c r="AY131" t="n">
         <v>-23.05593553629934</v>
@@ -34416,7 +34404,7 @@
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Pivô de alta</t>
         </is>
       </c>
       <c r="K133" t="n">
@@ -34451,7 +34439,7 @@
         <v>0</v>
       </c>
       <c r="V133" t="n">
-        <v>51848818688</v>
+        <v>51957202944</v>
       </c>
       <c r="W133" t="n">
         <v>40.6</v>
@@ -34519,10 +34507,14 @@
       </c>
       <c r="AS133" t="inlineStr"/>
       <c r="AT133" t="inlineStr"/>
-      <c r="AU133" t="inlineStr"/>
+      <c r="AU133" t="inlineStr">
+        <is>
+          <t>Pivô de alta</t>
+        </is>
+      </c>
       <c r="AV133" t="inlineStr">
         <is>
-          <t>Em Baixa</t>
+          <t>Lateral</t>
         </is>
       </c>
       <c r="AW133" t="n">
@@ -34538,14 +34530,14 @@
         <v>0</v>
       </c>
       <c r="BA133" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BB133" t="b">
         <v>0</v>
       </c>
       <c r="BC133" t="inlineStr">
         <is>
-          <t>sem sinal (-0.0% do topo; Em Baixa)</t>
+          <t>Pivô de alta</t>
         </is>
       </c>
     </row>
@@ -34685,7 +34677,7 @@
         <v>-35.41666472641126</v>
       </c>
       <c r="AY134" t="n">
-        <v>-89.31034509690564</v>
+        <v>-89.16083867989796</v>
       </c>
       <c r="AZ134" t="b">
         <v>0</v>

</xml_diff>